<commit_message>
Update the downloadable daily export
</commit_message>
<xml_diff>
--- a/public/daily_exports/macro_daily_export_2026-08-07.xlsx
+++ b/public/daily_exports/macro_daily_export_2026-08-07.xlsx
@@ -788,7 +788,7 @@
     <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="6" width="22" style="1" customWidth="1"/>
     <col min="7" max="7" width="25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="25" style="2" customWidth="1"/>
+    <col min="8" max="8" width="23" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -852,13 +852,13 @@
         <v>0.7030865550041199</v>
       </c>
       <c r="F4" s="12">
-        <v>0.7067137956619263</v>
+        <v>0.7069635987281799</v>
       </c>
       <c r="G4" s="12">
-        <v>0.0036272406578063965</v>
+        <v>0.0038770437240600586</v>
       </c>
       <c r="H4" s="13">
-        <v>0.005159024350544161</v>
+        <v>0.005514319249124711</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -878,13 +878,13 @@
         <v>0.7136485256714067</v>
       </c>
       <c r="F5" s="12">
-        <v>0.7176072117548339</v>
+        <v>0.7177978108069001</v>
       </c>
       <c r="G5" s="12">
-        <v>0.003958686083427199</v>
+        <v>0.004149285135493397</v>
       </c>
       <c r="H5" s="13">
-        <v>0.005547108893278807</v>
+        <v>0.005814185815895545</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -904,13 +904,13 @@
         <v>1.2312541817666498</v>
       </c>
       <c r="F6" s="12">
-        <v>1.238252071427264</v>
+        <v>1.2384360666442313</v>
       </c>
       <c r="G6" s="12">
-        <v>0.006997889660614209</v>
+        <v>0.007181884877581535</v>
       </c>
       <c r="H6" s="13">
-        <v>0.005683545903229614</v>
+        <v>0.0058329831353560735</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -930,13 +930,13 @@
         <v>1.152339220046997</v>
       </c>
       <c r="F7" s="12">
-        <v>1.156336784362793</v>
+        <v>1.1566041707992554</v>
       </c>
       <c r="G7" s="12">
-        <v>0.0039975643157958984</v>
+        <v>0.004264950752258301</v>
       </c>
       <c r="H7" s="13">
-        <v>0.0034690863994308874</v>
+        <v>0.0037011243547575567</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -956,13 +956,13 @@
         <v>1.3447909355163574</v>
       </c>
       <c r="F8" s="12">
-        <v>1.349800944328308</v>
+        <v>1.349892020225525</v>
       </c>
       <c r="G8" s="12">
-        <v>0.005010008811950684</v>
+        <v>0.0051010847091674805</v>
       </c>
       <c r="H8" s="13">
-        <v>0.003725492699002242</v>
+        <v>0.003793217647774183</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -982,13 +982,13 @@
         <v>0.006311059665976844</v>
       </c>
       <c r="F9" s="12">
-        <v>0.006341877681963195</v>
+        <v>0.006348884043352524</v>
       </c>
       <c r="G9" s="12">
-        <v>0.000030818015986351296</v>
+        <v>0.000037824377375679855</v>
       </c>
       <c r="H9" s="13">
-        <v>0.004883176141162515</v>
+        <v>0.005993348086945183</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1008,13 +1008,13 @@
         <v>0.5866134762763977</v>
       </c>
       <c r="F10" s="12">
-        <v>0.5892404317855835</v>
+        <v>0.5895531177520752</v>
       </c>
       <c r="G10" s="12">
-        <v>0.002626955509185791</v>
+        <v>0.0029396414756774902</v>
       </c>
       <c r="H10" s="13">
-        <v>0.004478171087818783</v>
+        <v>0.0050112068586238845</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1034,13 +1034,13 @@
         <v>99.94300079345703</v>
       </c>
       <c r="F11" s="12">
-        <v>99.55799865722656</v>
+        <v>99.56600189208984</v>
       </c>
       <c r="G11" s="12">
-        <v>-0.38500213623046875</v>
+        <v>-0.3769989013671875</v>
       </c>
       <c r="H11" s="13">
-        <v>-0.0038522170954834456</v>
+        <v>-0.003772139103030314</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1060,13 +1060,13 @@
         <v>4298.2998046875</v>
       </c>
       <c r="F12" s="12">
-        <v>4415.60009765625</v>
+        <v>4400.39990234375</v>
       </c>
       <c r="G12" s="12">
-        <v>117.30029296875</v>
+        <v>102.10009765625</v>
       </c>
       <c r="H12" s="13">
-        <v>0.027289928180632916</v>
+        <v>0.023753600794645502</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1086,13 +1086,13 @@
         <v>61.85499954223633</v>
       </c>
       <c r="F13" s="12">
-        <v>63.915000915527344</v>
+        <v>63.54999923706055</v>
       </c>
       <c r="G13" s="12">
-        <v>2.0600013732910156</v>
+        <v>1.6949996948242188</v>
       </c>
       <c r="H13" s="13">
-        <v>0.03330371657159881</v>
+        <v>0.027402792132700915</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1112,13 +1112,13 @@
         <v>78.16999816894531</v>
       </c>
       <c r="F14" s="12">
-        <v>78.13999938964844</v>
+        <v>78.43000030517578</v>
       </c>
       <c r="G14" s="12">
-        <v>-0.029998779296875</v>
+        <v>0.26000213623046875</v>
       </c>
       <c r="H14" s="13">
-        <v>-0.00038376333631273685</v>
+        <v>0.0033261115814349207</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1138,13 +1138,13 @@
         <v>83.33000183105469</v>
       </c>
       <c r="F15" s="12">
-        <v>83.30000305175781</v>
+        <v>83.75</v>
       </c>
       <c r="G15" s="12">
-        <v>-0.029998779296875</v>
+        <v>0.4199981689453125</v>
       </c>
       <c r="H15" s="13">
-        <v>-0.0003599997436420921</v>
+        <v>0.005040179523778665</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1164,13 +1164,13 @@
         <v>2.632999897003174</v>
       </c>
       <c r="F16" s="12">
-        <v>2.6700000762939453</v>
+        <v>2.6640000343322754</v>
       </c>
       <c r="G16" s="12">
-        <v>0.037000179290771484</v>
+        <v>0.031000137329101562</v>
       </c>
       <c r="H16" s="13">
-        <v>0.014052480341106177</v>
+        <v>0.011773694850647498</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1190,13 +1190,13 @@
         <v>6.7204999923706055</v>
       </c>
       <c r="F17" s="12">
-        <v>6.604499816894531</v>
+        <v>6.604000091552734</v>
       </c>
       <c r="G17" s="12">
-        <v>-0.11600017547607422</v>
+        <v>-0.1164999008178711</v>
       </c>
       <c r="H17" s="13">
-        <v>-0.017260646619710163</v>
+        <v>-0.017335004977327095</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1216,13 +1216,13 @@
         <v>461.75</v>
       </c>
       <c r="F18" s="12">
-        <v>464.5</v>
+        <v>465.75</v>
       </c>
       <c r="G18" s="12">
-        <v>2.75</v>
+        <v>4</v>
       </c>
       <c r="H18" s="13">
-        <v>0.005955603681645938</v>
+        <v>0.008662696264212233</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1242,13 +1242,13 @@
         <v>631</v>
       </c>
       <c r="F19" s="12">
-        <v>640.75</v>
+        <v>645</v>
       </c>
       <c r="G19" s="12">
-        <v>9.75</v>
+        <v>14</v>
       </c>
       <c r="H19" s="13">
-        <v>0.015451664025356582</v>
+        <v>0.022187004754358197</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1268,13 +1268,13 @@
         <v>1177.75</v>
       </c>
       <c r="F20" s="12">
-        <v>1178.75</v>
+        <v>1180.5</v>
       </c>
       <c r="G20" s="12">
-        <v>1</v>
+        <v>2.75</v>
       </c>
       <c r="H20" s="13">
-        <v>0.0008490766291657792</v>
+        <v>0.002334960730205893</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1294,13 +1294,13 @@
         <v>305.8500061035156</v>
       </c>
       <c r="F21" s="12">
-        <v>339.6000061035156</v>
+        <v>318.70001220703125</v>
       </c>
       <c r="G21" s="12">
-        <v>33.75</v>
+        <v>12.850006103515625</v>
       </c>
       <c r="H21" s="13">
-        <v>0.11034820770471798</v>
+        <v>0.0420140782968188</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1320,13 +1320,13 @@
         <v>5874</v>
       </c>
       <c r="F22" s="12">
-        <v>5910</v>
+        <v>5889</v>
       </c>
       <c r="G22" s="12">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="H22" s="13">
-        <v>0.006128702757916216</v>
+        <v>0.0025536261491316825</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update daily macro export
</commit_message>
<xml_diff>
--- a/public/daily_exports/macro_daily_export_2026-08-07.xlsx
+++ b/public/daily_exports/macro_daily_export_2026-08-07.xlsx
@@ -852,13 +852,13 @@
         <v>0.7030865550041199</v>
       </c>
       <c r="F4" s="12">
-        <v>0.7069635987281799</v>
+        <v>0.706813633441925</v>
       </c>
       <c r="G4" s="12">
-        <v>0.0038770437240600586</v>
+        <v>0.0037270784378051758</v>
       </c>
       <c r="H4" s="13">
-        <v>0.005514319249124711</v>
+        <v>0.005301023624016521</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -878,13 +878,13 @@
         <v>0.7136485256714067</v>
       </c>
       <c r="F5" s="12">
-        <v>0.7177978108069001</v>
+        <v>0.7176844462068703</v>
       </c>
       <c r="G5" s="12">
-        <v>0.004149285135493397</v>
+        <v>0.004035920535463644</v>
       </c>
       <c r="H5" s="13">
-        <v>0.005814185815895545</v>
+        <v>0.005655333669563278</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -904,13 +904,13 @@
         <v>1.2312541817666498</v>
       </c>
       <c r="F6" s="12">
-        <v>1.2384360666442313</v>
+        <v>1.2383287523066593</v>
       </c>
       <c r="G6" s="12">
-        <v>0.007181884877581535</v>
+        <v>0.007074570540009484</v>
       </c>
       <c r="H6" s="13">
-        <v>0.0058329831353560735</v>
+        <v>0.005745824578527348</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -930,13 +930,13 @@
         <v>1.152339220046997</v>
       </c>
       <c r="F7" s="12">
-        <v>1.1566041707992554</v>
+        <v>1.156336784362793</v>
       </c>
       <c r="G7" s="12">
-        <v>0.004264950752258301</v>
+        <v>0.0039975643157958984</v>
       </c>
       <c r="H7" s="13">
-        <v>0.0037011243547575567</v>
+        <v>0.0034690863994308874</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -956,13 +956,13 @@
         <v>1.3447909355163574</v>
       </c>
       <c r="F8" s="12">
-        <v>1.349892020225525</v>
+        <v>1.3497462272644043</v>
       </c>
       <c r="G8" s="12">
-        <v>0.0051010847091674805</v>
+        <v>0.004955291748046875</v>
       </c>
       <c r="H8" s="13">
-        <v>0.003793217647774183</v>
+        <v>0.0036848045426065568</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -982,13 +982,13 @@
         <v>0.006311059665976844</v>
       </c>
       <c r="F9" s="12">
-        <v>0.006348884043352524</v>
+        <v>0.006351787205824229</v>
       </c>
       <c r="G9" s="12">
-        <v>0.000037824377375679855</v>
+        <v>0.000040727539847385495</v>
       </c>
       <c r="H9" s="13">
-        <v>0.005993348086945183</v>
+        <v>0.006453359974862627</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1008,13 +1008,13 @@
         <v>0.5866134762763977</v>
       </c>
       <c r="F10" s="12">
-        <v>0.5895531177520752</v>
+        <v>0.5893446803092957</v>
       </c>
       <c r="G10" s="12">
-        <v>0.0029396414756774902</v>
+        <v>0.0027312040328979492</v>
       </c>
       <c r="H10" s="13">
-        <v>0.0050112068586238845</v>
+        <v>0.004655883547433293</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1034,13 +1034,13 @@
         <v>99.94300079345703</v>
       </c>
       <c r="F11" s="12">
-        <v>99.56600189208984</v>
+        <v>99.54199981689453</v>
       </c>
       <c r="G11" s="12">
-        <v>-0.3769989013671875</v>
+        <v>-0.4010009765625</v>
       </c>
       <c r="H11" s="13">
-        <v>-0.003772139103030314</v>
+        <v>-0.004012296742932575</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1060,13 +1060,13 @@
         <v>4298.2998046875</v>
       </c>
       <c r="F12" s="12">
-        <v>4400.39990234375</v>
+        <v>4393.7998046875</v>
       </c>
       <c r="G12" s="12">
-        <v>102.10009765625</v>
+        <v>95.5</v>
       </c>
       <c r="H12" s="13">
-        <v>0.023753600794645502</v>
+        <v>0.022218087229711747</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1086,13 +1086,13 @@
         <v>61.85499954223633</v>
       </c>
       <c r="F13" s="12">
-        <v>63.54999923706055</v>
+        <v>63.380001068115234</v>
       </c>
       <c r="G13" s="12">
-        <v>1.6949996948242188</v>
+        <v>1.5250015258789062</v>
       </c>
       <c r="H13" s="13">
-        <v>0.027402792132700915</v>
+        <v>0.02465445860746618</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1112,13 +1112,13 @@
         <v>78.16999816894531</v>
       </c>
       <c r="F14" s="12">
-        <v>78.43000030517578</v>
+        <v>78.22000122070312</v>
       </c>
       <c r="G14" s="12">
-        <v>0.26000213623046875</v>
+        <v>0.0500030517578125</v>
       </c>
       <c r="H14" s="13">
-        <v>0.0033261115814349207</v>
+        <v>0.0006396706272109309</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1135,17 +1135,15 @@
         <v>36</v>
       </c>
       <c r="E15" s="12">
-        <v>83.33000183105469</v>
+        <v>0</v>
       </c>
       <c r="F15" s="12">
-        <v>83.75</v>
+        <v>83.52999877929688</v>
       </c>
       <c r="G15" s="12">
-        <v>0.4199981689453125</v>
-      </c>
-      <c r="H15" s="13">
-        <v>0.005040179523778665</v>
-      </c>
+        <v>83.52999877929688</v>
+      </c>
+      <c r="H15" s="2"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
@@ -1164,13 +1162,13 @@
         <v>2.632999897003174</v>
       </c>
       <c r="F16" s="12">
-        <v>2.6640000343322754</v>
+        <v>2.6700000762939453</v>
       </c>
       <c r="G16" s="12">
-        <v>0.031000137329101562</v>
+        <v>0.037000179290771484</v>
       </c>
       <c r="H16" s="13">
-        <v>0.011773694850647498</v>
+        <v>0.014052480341106177</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1190,13 +1188,13 @@
         <v>6.7204999923706055</v>
       </c>
       <c r="F17" s="12">
-        <v>6.604000091552734</v>
+        <v>6.5879998207092285</v>
       </c>
       <c r="G17" s="12">
-        <v>-0.1164999008178711</v>
+        <v>-0.13250017166137695</v>
       </c>
       <c r="H17" s="13">
-        <v>-0.017335004977327095</v>
+        <v>-0.01971582052106191</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1216,13 +1214,13 @@
         <v>461.75</v>
       </c>
       <c r="F18" s="12">
-        <v>465.75</v>
+        <v>464.25</v>
       </c>
       <c r="G18" s="12">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="H18" s="13">
-        <v>0.008662696264212233</v>
+        <v>0.00541418516513259</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1242,13 +1240,13 @@
         <v>631</v>
       </c>
       <c r="F19" s="12">
-        <v>645</v>
+        <v>641.5</v>
       </c>
       <c r="G19" s="12">
-        <v>14</v>
+        <v>10.5</v>
       </c>
       <c r="H19" s="13">
-        <v>0.022187004754358197</v>
+        <v>0.016640253565768592</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1268,13 +1266,13 @@
         <v>1177.75</v>
       </c>
       <c r="F20" s="12">
-        <v>1180.5</v>
+        <v>1177.75</v>
       </c>
       <c r="G20" s="12">
-        <v>2.75</v>
+        <v>0</v>
       </c>
       <c r="H20" s="13">
-        <v>0.002334960730205893</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1294,13 +1292,13 @@
         <v>305.8500061035156</v>
       </c>
       <c r="F21" s="12">
-        <v>318.70001220703125</v>
+        <v>315.6000061035156</v>
       </c>
       <c r="G21" s="12">
-        <v>12.850006103515625</v>
+        <v>9.75</v>
       </c>
       <c r="H21" s="13">
-        <v>0.0420140782968188</v>
+        <v>0.03187837111469638</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1320,13 +1318,13 @@
         <v>5874</v>
       </c>
       <c r="F22" s="12">
-        <v>5889</v>
+        <v>5855</v>
       </c>
       <c r="G22" s="12">
-        <v>15</v>
+        <v>-19</v>
       </c>
       <c r="H22" s="13">
-        <v>0.0025536261491316825</v>
+        <v>-0.00323459312223362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>